<commit_message>
BL node presentation: map anchored BL tools to their nodes, expand framework BL tools chain-wide
- data/: canonical e520ec18 (ZH) / d8538e34 (EN) — BL node-mapping batch
  (BL-3/BL-4 tools -> N7, BL-6 -> N2, BL-7:T01 -> N15; sheet5 rebuilt 144->145 edges)
- generator: BL-track tools whose only node mapping is 0 now expand to all 15 nodes
  (framework regimes apply chain-wide); non-BL 0-node tools unchanged
- guide: chain-wide presentation note (ZH+EN); README: BL presentation rule
- verified locally: BL-only filter shows 15 on every node, N2=16 / N7=18 / N15=16

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/US-overseas-AI-compute-controls_v2_EN.xlsx
+++ b/data/US-overseas-AI-compute-controls_v2_EN.xlsx
@@ -4147,7 +4147,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N15</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4367,7 +4367,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N2</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -22163,7 +22163,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N15</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -22282,7 +22282,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N2</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -22299,7 +22299,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -22319,7 +22319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B145"/>
+  <dimension ref="A1:B146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23218,7 +23218,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23230,7 +23230,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23254,7 +23254,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N2</t>
         </is>
       </c>
     </row>
@@ -23273,19 +23273,19 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BL-8</t>
+          <t>BL-7</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N15</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BL-9</t>
+          <t>BL-8</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -23297,24 +23297,24 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>C-1</t>
+          <t>BL-9</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>C-2</t>
+          <t>C-1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -23326,14 +23326,14 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>C-3</t>
+          <t>C-2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -23350,31 +23350,31 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>D-1</t>
+          <t>C-3</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>N14</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>E-1</t>
+          <t>D-1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>N5</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -23386,19 +23386,19 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>N6</t>
+          <t>N5</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>E-2</t>
+          <t>E-1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>N6</t>
         </is>
       </c>
     </row>
@@ -23410,19 +23410,19 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>E-3</t>
+          <t>E-2</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23434,7 +23434,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23446,19 +23446,19 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N13</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>E-4</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N14</t>
         </is>
       </c>
     </row>
@@ -23470,7 +23470,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23482,19 +23482,19 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>E-5</t>
+          <t>E-4</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23506,7 +23506,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>N2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23518,19 +23518,19 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>N5</t>
+          <t>N2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>E-6</t>
+          <t>E-5</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>N5</t>
         </is>
       </c>
     </row>
@@ -23542,7 +23542,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>N1</t>
         </is>
       </c>
     </row>
@@ -23554,7 +23554,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
@@ -23566,7 +23566,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -23578,7 +23578,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N13</t>
         </is>
       </c>
     </row>
@@ -23590,7 +23590,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>N2</t>
+          <t>N14</t>
         </is>
       </c>
     </row>
@@ -23602,7 +23602,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>N5</t>
+          <t>N2</t>
         </is>
       </c>
     </row>
@@ -23614,7 +23614,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>N6</t>
+          <t>N5</t>
         </is>
       </c>
     </row>
@@ -23626,19 +23626,19 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N6</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>E-7</t>
+          <t>E-6</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23662,7 +23662,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -23674,19 +23674,19 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N13</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>E-8</t>
+          <t>E-7</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N14</t>
         </is>
       </c>
     </row>
@@ -23698,7 +23698,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23710,7 +23710,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>N2</t>
+          <t>N1</t>
         </is>
       </c>
     </row>
@@ -23722,7 +23722,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>N3</t>
+          <t>N2</t>
         </is>
       </c>
     </row>
@@ -23734,7 +23734,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>N5</t>
+          <t>N3</t>
         </is>
       </c>
     </row>
@@ -23746,26 +23746,26 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>N6</t>
+          <t>N5</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>F-1</t>
+          <t>E-8</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N6</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -23777,7 +23777,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>F-2</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -23789,7 +23789,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>F-3</t>
+          <t>F-2</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -23801,12 +23801,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>F-4</t>
+          <t>F-3</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23818,31 +23818,31 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>F-6</t>
+          <t>F-4</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>F-7</t>
+          <t>F-6</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>N2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23854,7 +23854,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>N5</t>
+          <t>N2</t>
         </is>
       </c>
     </row>
@@ -23866,26 +23866,26 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N5</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>F-8</t>
+          <t>F-7</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>F-9</t>
+          <t>F-8</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -23902,19 +23902,19 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>G-1a</t>
+          <t>F-9</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -23926,7 +23926,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -23938,7 +23938,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
@@ -23950,7 +23950,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -23962,7 +23962,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N13</t>
         </is>
       </c>
     </row>
@@ -23974,7 +23974,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>N15</t>
+          <t>N14</t>
         </is>
       </c>
     </row>
@@ -23986,19 +23986,19 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>N7</t>
+          <t>N15</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>G-1b</t>
+          <t>G-1a</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N7</t>
         </is>
       </c>
     </row>
@@ -24010,7 +24010,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24022,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>N11</t>
         </is>
       </c>
     </row>
@@ -24034,7 +24034,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>N12</t>
         </is>
       </c>
     </row>
@@ -24046,7 +24046,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N13</t>
         </is>
       </c>
     </row>
@@ -24057,6 +24057,18 @@
         </is>
       </c>
       <c r="B145" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>G-1b</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
         <is>
           <t>N7</t>
         </is>

</xml_diff>